<commit_message>
Fix #NAME? errors: replace dot-notation functions with compatible equivalents in 04_Correlation_Covariance.xlsx
</commit_message>
<xml_diff>
--- a/rFLA300/chapter-12/04_Correlation_Covariance.xlsx
+++ b/rFLA300/chapter-12/04_Correlation_Covariance.xlsx
@@ -113,7 +113,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -127,11 +127,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -221,6 +249,8 @@
     <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -612,6 +642,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -913,6 +944,7 @@
         <v>24</v>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
@@ -959,23 +991,23 @@
         </is>
       </c>
       <c r="B20" s="11">
-        <f>COVARIANCE.S(B5:B16,C5:C16)</f>
+        <f>_xlfn.COVARIANCE.S(B5:B16,C5:C16)</f>
         <v/>
       </c>
       <c r="C20" s="11">
-        <f>COVARIANCE.S(B5:B16,E5:E16)</f>
+        <f>_xlfn.COVARIANCE.S(B5:B16,E5:E16)</f>
         <v/>
       </c>
       <c r="D20" s="11">
-        <f>COVARIANCE.S(D5:D16,C5:C16)</f>
+        <f>_xlfn.COVARIANCE.S(D5:D16,C5:C16)</f>
         <v/>
       </c>
       <c r="E20" s="11">
-        <f>COVARIANCE.S(D5:D16,F5:F16)</f>
+        <f>_xlfn.COVARIANCE.S(D5:D16,F5:F16)</f>
         <v/>
       </c>
       <c r="F20" s="11">
-        <f>COVARIANCE.S(C5:C16,F5:F16)</f>
+        <f>_xlfn.COVARIANCE.S(C5:C16,F5:F16)</f>
         <v/>
       </c>
     </row>
@@ -1033,6 +1065,7 @@
         <v/>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
@@ -1056,7 +1089,8 @@
           <t>What It Means</t>
         </is>
       </c>
-      <c r="D25" s="16" t="n"/>
+      <c r="D25" s="31" t="n"/>
+      <c r="E25" s="32" t="n"/>
       <c r="F25" s="17" t="inlineStr">
         <is>
           <t>Example</t>
@@ -1079,7 +1113,8 @@
           <t>As X increases, Y almost always increases proportionally.</t>
         </is>
       </c>
-      <c r="D26" s="16" t="n"/>
+      <c r="D26" s="31" t="n"/>
+      <c r="E26" s="32" t="n"/>
       <c r="F26" s="4" t="inlineStr">
         <is>
           <t>Ad spend &amp; revenue — reliable predictor.</t>
@@ -1102,7 +1137,8 @@
           <t>Clear positive relationship with some scatter.</t>
         </is>
       </c>
-      <c r="D27" s="16" t="n"/>
+      <c r="D27" s="31" t="n"/>
+      <c r="E27" s="32" t="n"/>
       <c r="F27" s="24" t="inlineStr">
         <is>
           <t>Temperature &amp; traffic.</t>
@@ -1125,7 +1161,8 @@
           <t>Some relationship, but other factors matter too.</t>
         </is>
       </c>
-      <c r="D28" s="16" t="n"/>
+      <c r="D28" s="31" t="n"/>
+      <c r="E28" s="32" t="n"/>
       <c r="F28" s="4" t="inlineStr">
         <is>
           <t>Web visits &amp; sales.</t>
@@ -1148,7 +1185,8 @@
           <t>Very little linear relationship.</t>
         </is>
       </c>
-      <c r="D29" s="16" t="n"/>
+      <c r="D29" s="31" t="n"/>
+      <c r="E29" s="32" t="n"/>
       <c r="F29" s="24" t="inlineStr">
         <is>
           <t>Shoe size &amp; test scores.</t>
@@ -1171,7 +1209,8 @@
           <t>As X increases, Y tends to decrease.</t>
         </is>
       </c>
-      <c r="D30" s="16" t="n"/>
+      <c r="D30" s="31" t="n"/>
+      <c r="E30" s="32" t="n"/>
       <c r="F30" s="4" t="inlineStr">
         <is>
           <t>Price &amp; quantity demanded.</t>
@@ -1194,7 +1233,8 @@
           <t>Clear negative relationship.</t>
         </is>
       </c>
-      <c r="D31" s="16" t="n"/>
+      <c r="D31" s="31" t="n"/>
+      <c r="E31" s="32" t="n"/>
       <c r="F31" s="24" t="inlineStr">
         <is>
           <t>Study time &amp; exam errors.</t>
@@ -1217,13 +1257,16 @@
           <t>Almost perfect inverse relationship.</t>
         </is>
       </c>
-      <c r="D32" s="16" t="n"/>
+      <c r="D32" s="31" t="n"/>
+      <c r="E32" s="32" t="n"/>
       <c r="F32" s="4" t="inlineStr">
         <is>
           <t>Hours worked &amp; time available.</t>
         </is>
       </c>
     </row>
+    <row r="33"/>
+    <row r="34"/>
     <row r="35" ht="40" customHeight="1">
       <c r="A35" s="25" t="inlineStr">
         <is>
@@ -1292,6 +1335,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1588,6 +1632,7 @@
         <v>24</v>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
@@ -1753,6 +1798,8 @@
         <v>1</v>
       </c>
     </row>
+    <row r="25"/>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
@@ -1802,6 +1849,7 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
     <row r="35" ht="40" customHeight="1">
       <c r="A35" s="30" t="inlineStr">
         <is>

</xml_diff>